<commit_message>
Minor powers and chapters changes
</commit_message>
<xml_diff>
--- a/src/resources/horde_cards.xlsx
+++ b/src/resources/horde_cards.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dsaban/git/perso/windwalkers-cardgame/src/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C52FABD-63DC-F64C-BC69-94A122BAB472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF051C5A-07D0-7245-AC65-4AC170CD20A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="760" windowWidth="28920" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-140" yWindow="1160" windowWidth="28920" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -772,9 +785,6 @@
     <t>Son sourire est divin et son visage angélique. Benelim est responsable des affaires du pack.</t>
   </si>
   <si>
-    <t>:discard:: Lancez +1 :d6-blue-violet: / :card: &lt;b&gt;PACK&lt;/b&gt;.</t>
-  </si>
-  <si>
     <t>Benelim.png</t>
   </si>
   <si>
@@ -969,10 +979,6 @@
     <t>Usmos était le gardien du fameux Harem d’Alticcio. Depuis qu’il s’est affranchi, il a décidé de libérer les esclaves qu’il rencontre.</t>
   </si>
   <si>
-    <t>:tap:: Utilisez un pouvoir :card: &lt;b&gt;TRAÎNE&lt;/b&gt; sans :discard:.
-:tap: ce :card:&lt;b&gt;TRAÎNE&lt;/b&gt;</t>
-  </si>
-  <si>
     <t>Usmos.png</t>
   </si>
   <si>
@@ -1031,9 +1037,6 @@
   </si>
   <si>
     <t>Eclaireuse chevronnée, connue pour sa capacité à rallier des alliés où qu’ils se trouvent.</t>
-  </si>
-  <si>
-    <t>:tap:: :tuile: villages = :tuile: villes: Ignorez tous :d6-black-white-green: et vous recrutez tout type de :card: Si :rest-all: gagnez  +1 :moral:</t>
   </si>
   <si>
     <t>Lyara.png</t>
@@ -1346,9 +1349,6 @@
     <t>Et pourquoi pas un Dragon ?</t>
   </si>
   <si>
-    <t>:tap:: :tap: 1 autre :card: et gagnez +4 :moral:</t>
-  </si>
-  <si>
     <t>Dragon.png</t>
   </si>
   <si>
@@ -1475,10 +1475,6 @@
     <t>Le seul obstacle insurmontable, c’est votre propre peur. Barakiel ne connaît pas la peur.</t>
   </si>
   <si>
-    <t>:discard:: Tous les :d6-black: sont :d6-green: et les :d6-violet: sont :d6-blue:
-:force-x: ⮕ :force-1:</t>
-  </si>
-  <si>
     <t>Barakiel.png</t>
   </si>
   <si>
@@ -1558,9 +1554,6 @@
   </si>
   <si>
     <t>Les frères Torantor sont des valeurs sûres, solides et bienveillants.</t>
-  </si>
-  <si>
-    <t>:discard:: Lancez +1 :d6-violet:, :rest: 1 autre :card: &lt;b&gt;Torantor&lt;/b&gt;.</t>
   </si>
   <si>
     <t>Zaffa.png</t>
@@ -1714,6 +1707,24 @@
   </si>
   <si>
     <t>Trumpette.png</t>
+  </si>
+  <si>
+    <t>:tap:: :tap: 1 autre :card: et gagnez +3 :moral:</t>
+  </si>
+  <si>
+    <t>:discard:: Lancez +1 :d6-blue: / :card: &lt;b&gt;PACK&lt;/b&gt;.</t>
+  </si>
+  <si>
+    <t>:discard:: Lancez +2 :d6-violet:, :rest: 1 autre :card: &lt;b&gt;Torantor&lt;/b&gt;.</t>
+  </si>
+  <si>
+    <t>:discard:: Tous les :d6-black: sont :d6-green: et les :d6-violet: sont :d6-blue:</t>
+  </si>
+  <si>
+    <t>:tap:: :tuile: villages = :tuile: villes: Ignorez tous :d6-black-white-green: et vous recrutez tout type de :card:</t>
+  </si>
+  <si>
+    <t>:tap:: :tap: :card: &lt;b&gt;TRAÎNE&lt;/b&gt; pour utiliser son pouvoir.</t>
   </si>
 </sst>
 </file>
@@ -4053,13 +4064,13 @@
         <v>245</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>246</v>
+        <v>551</v>
       </c>
       <c r="H43">
         <v>3</v>
       </c>
       <c r="I43" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L43" t="s">
         <v>46</v>
@@ -4079,10 +4090,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>247</v>
+      </c>
+      <c r="C44" t="s">
         <v>248</v>
-      </c>
-      <c r="C44" t="s">
-        <v>249</v>
       </c>
       <c r="D44" t="s">
         <v>28</v>
@@ -4091,16 +4102,16 @@
         <v>180</v>
       </c>
       <c r="F44" t="s">
+        <v>249</v>
+      </c>
+      <c r="G44" s="3" t="s">
         <v>250</v>
-      </c>
-      <c r="G44" s="3" t="s">
-        <v>251</v>
       </c>
       <c r="H44">
         <v>2</v>
       </c>
       <c r="I44" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="L44" t="s">
         <v>57</v>
@@ -4120,10 +4131,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>252</v>
+      </c>
+      <c r="C45" t="s">
         <v>253</v>
-      </c>
-      <c r="C45" t="s">
-        <v>254</v>
       </c>
       <c r="D45" t="s">
         <v>36</v>
@@ -4132,16 +4143,16 @@
         <v>180</v>
       </c>
       <c r="F45" t="s">
+        <v>254</v>
+      </c>
+      <c r="G45" s="3" t="s">
         <v>255</v>
-      </c>
-      <c r="G45" s="3" t="s">
-        <v>256</v>
       </c>
       <c r="H45">
         <v>2</v>
       </c>
       <c r="I45" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="M45" t="s">
         <v>46</v>
@@ -4155,10 +4166,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C46" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D46" t="s">
         <v>36</v>
@@ -4167,16 +4178,16 @@
         <v>180</v>
       </c>
       <c r="F46" t="s">
+        <v>258</v>
+      </c>
+      <c r="G46" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="H46">
         <v>3</v>
       </c>
       <c r="I46" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L46" t="s">
         <v>33</v>
@@ -4196,10 +4207,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C47" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
@@ -4208,16 +4219,16 @@
         <v>180</v>
       </c>
       <c r="F47" t="s">
+        <v>262</v>
+      </c>
+      <c r="G47" s="3" t="s">
         <v>263</v>
-      </c>
-      <c r="G47" s="3" t="s">
-        <v>264</v>
       </c>
       <c r="H47">
         <v>2</v>
       </c>
       <c r="I47" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="M47" t="s">
         <v>107</v>
@@ -4234,10 +4245,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
+        <v>265</v>
+      </c>
+      <c r="C48" t="s">
         <v>266</v>
-      </c>
-      <c r="C48" t="s">
-        <v>267</v>
       </c>
       <c r="D48" t="s">
         <v>28</v>
@@ -4246,16 +4257,16 @@
         <v>180</v>
       </c>
       <c r="F48" t="s">
+        <v>267</v>
+      </c>
+      <c r="G48" s="3" t="s">
         <v>268</v>
-      </c>
-      <c r="G48" s="3" t="s">
-        <v>269</v>
       </c>
       <c r="H48">
         <v>2</v>
       </c>
       <c r="I48" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="L48" t="s">
         <v>46</v>
@@ -4272,10 +4283,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
+        <v>270</v>
+      </c>
+      <c r="C49" t="s">
         <v>271</v>
-      </c>
-      <c r="C49" t="s">
-        <v>272</v>
       </c>
       <c r="D49" t="s">
         <v>36</v>
@@ -4284,16 +4295,16 @@
         <v>180</v>
       </c>
       <c r="F49" t="s">
+        <v>272</v>
+      </c>
+      <c r="G49" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="G49" s="3" t="s">
+      <c r="H49">
+        <v>1</v>
+      </c>
+      <c r="I49" t="s">
         <v>274</v>
-      </c>
-      <c r="H49">
-        <v>1</v>
-      </c>
-      <c r="I49" t="s">
-        <v>275</v>
       </c>
       <c r="M49" t="s">
         <v>33</v>
@@ -4310,10 +4321,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C50" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D50" t="s">
         <v>36</v>
@@ -4322,16 +4333,16 @@
         <v>180</v>
       </c>
       <c r="F50" t="s">
+        <v>276</v>
+      </c>
+      <c r="G50" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="G50" s="3" t="s">
+      <c r="H50">
+        <v>1</v>
+      </c>
+      <c r="I50" t="s">
         <v>278</v>
-      </c>
-      <c r="H50">
-        <v>1</v>
-      </c>
-      <c r="I50" t="s">
-        <v>279</v>
       </c>
       <c r="M50" t="s">
         <v>33</v>
@@ -4351,10 +4362,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C51" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D51" t="s">
         <v>28</v>
@@ -4363,16 +4374,16 @@
         <v>180</v>
       </c>
       <c r="F51" t="s">
+        <v>280</v>
+      </c>
+      <c r="G51" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="G51" s="3" t="s">
+      <c r="H51">
+        <v>1</v>
+      </c>
+      <c r="I51" t="s">
         <v>282</v>
-      </c>
-      <c r="H51">
-        <v>1</v>
-      </c>
-      <c r="I51" t="s">
-        <v>283</v>
       </c>
       <c r="L51" t="s">
         <v>40</v>
@@ -4389,10 +4400,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>283</v>
+      </c>
+      <c r="C52" t="s">
         <v>284</v>
-      </c>
-      <c r="C52" t="s">
-        <v>285</v>
       </c>
       <c r="D52" t="s">
         <v>36</v>
@@ -4401,16 +4412,16 @@
         <v>180</v>
       </c>
       <c r="F52" t="s">
+        <v>285</v>
+      </c>
+      <c r="G52" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>287</v>
       </c>
       <c r="H52">
         <v>3</v>
       </c>
       <c r="I52" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="K52" t="s">
         <v>52</v>
@@ -4433,10 +4444,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>288</v>
+      </c>
+      <c r="C53" t="s">
         <v>289</v>
-      </c>
-      <c r="C53" t="s">
-        <v>290</v>
       </c>
       <c r="D53" t="s">
         <v>28</v>
@@ -4445,16 +4456,16 @@
         <v>180</v>
       </c>
       <c r="F53" t="s">
+        <v>290</v>
+      </c>
+      <c r="G53" s="3" t="s">
         <v>291</v>
-      </c>
-      <c r="G53" s="3" t="s">
-        <v>292</v>
       </c>
       <c r="H53">
         <v>3</v>
       </c>
       <c r="I53" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K53" t="s">
         <v>52</v>
@@ -4477,10 +4488,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>293</v>
+      </c>
+      <c r="C54" t="s">
         <v>294</v>
-      </c>
-      <c r="C54" t="s">
-        <v>295</v>
       </c>
       <c r="D54" t="s">
         <v>28</v>
@@ -4489,16 +4500,16 @@
         <v>180</v>
       </c>
       <c r="F54" t="s">
+        <v>295</v>
+      </c>
+      <c r="G54" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="G54" s="3" t="s">
+      <c r="H54">
+        <v>1</v>
+      </c>
+      <c r="I54" t="s">
         <v>297</v>
-      </c>
-      <c r="H54">
-        <v>1</v>
-      </c>
-      <c r="I54" t="s">
-        <v>298</v>
       </c>
       <c r="U54">
         <v>1</v>
@@ -4512,10 +4523,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>298</v>
+      </c>
+      <c r="C55" t="s">
         <v>299</v>
-      </c>
-      <c r="C55" t="s">
-        <v>300</v>
       </c>
       <c r="D55" t="s">
         <v>36</v>
@@ -4524,16 +4535,16 @@
         <v>180</v>
       </c>
       <c r="F55" t="s">
+        <v>300</v>
+      </c>
+      <c r="G55" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="G55" s="3" t="s">
-        <v>302</v>
       </c>
       <c r="H55">
         <v>3</v>
       </c>
       <c r="I55" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="M55" t="s">
         <v>128</v>
@@ -4550,7 +4561,7 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C56" t="s">
         <v>48</v>
@@ -4562,19 +4573,19 @@
         <v>29</v>
       </c>
       <c r="F56" t="s">
+        <v>304</v>
+      </c>
+      <c r="G56" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>306</v>
       </c>
       <c r="H56">
         <v>2</v>
       </c>
       <c r="I56" t="s">
+        <v>306</v>
+      </c>
+      <c r="J56" t="s">
         <v>307</v>
-      </c>
-      <c r="J56" t="s">
-        <v>308</v>
       </c>
       <c r="M56" t="s">
         <v>128</v>
@@ -4588,7 +4599,7 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C57" t="s">
         <v>48</v>
@@ -4600,16 +4611,16 @@
         <v>29</v>
       </c>
       <c r="F57" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>311</v>
+        <v>555</v>
       </c>
       <c r="H57">
         <v>3</v>
       </c>
       <c r="I57" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="M57" t="s">
         <v>212</v>
@@ -4626,7 +4637,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C58" t="s">
         <v>42</v>
@@ -4638,16 +4649,16 @@
         <v>29</v>
       </c>
       <c r="F58" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H58">
         <v>2</v>
       </c>
       <c r="I58" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="M58" t="s">
         <v>64</v>
@@ -4664,10 +4675,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C59" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D59" t="s">
         <v>36</v>
@@ -4676,16 +4687,16 @@
         <v>29</v>
       </c>
       <c r="F59" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="M59" t="s">
         <v>107</v>
@@ -4708,7 +4719,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C60" t="s">
         <v>48</v>
@@ -4720,19 +4731,19 @@
         <v>29</v>
       </c>
       <c r="F60" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H60">
         <v>2</v>
       </c>
       <c r="I60" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J60" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="61" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -4740,7 +4751,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C61" t="s">
         <v>42</v>
@@ -4752,16 +4763,16 @@
         <v>29</v>
       </c>
       <c r="F61" t="s">
+        <v>325</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="H61">
+        <v>1</v>
+      </c>
+      <c r="I61" t="s">
         <v>327</v>
-      </c>
-      <c r="G61" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="H61">
-        <v>1</v>
-      </c>
-      <c r="I61" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="62" spans="1:26" ht="80" customHeight="1" x14ac:dyDescent="0.2">
@@ -4769,7 +4780,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C62" t="s">
         <v>42</v>
@@ -4781,16 +4792,16 @@
         <v>29</v>
       </c>
       <c r="F62" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>332</v>
+        <v>554</v>
       </c>
       <c r="H62">
         <v>1</v>
       </c>
       <c r="I62" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="63" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -4798,7 +4809,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="C63" t="s">
         <v>169</v>
@@ -4810,16 +4821,16 @@
         <v>60</v>
       </c>
       <c r="F63" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="H63">
         <v>1</v>
       </c>
       <c r="I63" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="M63" t="s">
         <v>212</v>
@@ -4839,10 +4850,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C64" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="D64" t="s">
         <v>36</v>
@@ -4851,16 +4862,16 @@
         <v>60</v>
       </c>
       <c r="F64" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="H64">
         <v>1</v>
       </c>
       <c r="I64" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="M64" t="s">
         <v>212</v>
@@ -4886,10 +4897,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C65" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="D65" t="s">
         <v>28</v>
@@ -4898,16 +4909,16 @@
         <v>60</v>
       </c>
       <c r="F65" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="H65">
         <v>1</v>
       </c>
       <c r="I65" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="M65" t="s">
         <v>107</v>
@@ -4933,10 +4944,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C66" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="D66" t="s">
         <v>28</v>
@@ -4945,16 +4956,16 @@
         <v>60</v>
       </c>
       <c r="F66" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="H66">
         <v>1</v>
       </c>
       <c r="I66" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="N66">
         <v>1</v>
@@ -4977,10 +4988,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C67" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="D67" t="s">
         <v>28</v>
@@ -4989,16 +5000,16 @@
         <v>60</v>
       </c>
       <c r="F67" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="H67">
         <v>1</v>
       </c>
       <c r="I67" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="M67" t="s">
         <v>128</v>
@@ -5013,7 +5024,7 @@
         <v>0</v>
       </c>
       <c r="Z67" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="68" spans="1:26" ht="64" customHeight="1" x14ac:dyDescent="0.2">
@@ -5021,10 +5032,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C68" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="D68" t="s">
         <v>28</v>
@@ -5033,16 +5044,16 @@
         <v>60</v>
       </c>
       <c r="F68" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="H68">
         <v>1</v>
       </c>
       <c r="I68" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="M68" t="s">
         <v>128</v>
@@ -5057,7 +5068,7 @@
         <v>0</v>
       </c>
       <c r="Z68" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="69" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -5065,10 +5076,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C69" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="D69" t="s">
         <v>28</v>
@@ -5077,16 +5088,16 @@
         <v>60</v>
       </c>
       <c r="F69" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="H69">
         <v>2</v>
       </c>
       <c r="I69" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="M69" t="s">
         <v>33</v>
@@ -5109,10 +5120,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C70" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="D70" t="s">
         <v>28</v>
@@ -5121,16 +5132,16 @@
         <v>60</v>
       </c>
       <c r="F70" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="H70">
         <v>1</v>
       </c>
       <c r="I70" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="M70" t="s">
         <v>212</v>
@@ -5148,7 +5159,7 @@
         <v>0</v>
       </c>
       <c r="Z70" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="71" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -5156,10 +5167,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C71" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="D71" t="s">
         <v>28</v>
@@ -5168,16 +5179,16 @@
         <v>60</v>
       </c>
       <c r="F71" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H71">
         <v>3</v>
       </c>
       <c r="I71" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="M71" t="s">
         <v>33</v>
@@ -5192,7 +5203,7 @@
         <v>1</v>
       </c>
       <c r="Z71" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="72" spans="1:26" ht="80" customHeight="1" x14ac:dyDescent="0.2">
@@ -5200,10 +5211,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C72" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="D72" t="s">
         <v>36</v>
@@ -5212,19 +5223,19 @@
         <v>60</v>
       </c>
       <c r="F72" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="H72">
         <v>3</v>
       </c>
       <c r="I72" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="J72" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="73" spans="1:26" ht="80" customHeight="1" x14ac:dyDescent="0.2">
@@ -5232,10 +5243,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C73" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D73" t="s">
         <v>28</v>
@@ -5244,19 +5255,19 @@
         <v>60</v>
       </c>
       <c r="F73" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="H73">
         <v>2</v>
       </c>
       <c r="I73" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="J73" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="X73">
         <v>1</v>
@@ -5267,10 +5278,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C74" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="D74" t="s">
         <v>28</v>
@@ -5279,19 +5290,19 @@
         <v>60</v>
       </c>
       <c r="F74" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="H74">
         <v>2</v>
       </c>
       <c r="I74" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="J74" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="75" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -5299,10 +5310,10 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="C75" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="D75" t="s">
         <v>36</v>
@@ -5311,16 +5322,16 @@
         <v>130</v>
       </c>
       <c r="F75" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="H75">
         <v>2</v>
       </c>
       <c r="I75" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="M75" t="s">
         <v>64</v>
@@ -5346,7 +5357,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="C76" t="s">
         <v>35</v>
@@ -5358,16 +5369,16 @@
         <v>130</v>
       </c>
       <c r="F76" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H76">
         <v>3</v>
       </c>
       <c r="I76" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="M76" t="s">
         <v>52</v>
@@ -5390,10 +5401,10 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C77" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="D77" t="s">
         <v>36</v>
@@ -5402,16 +5413,16 @@
         <v>130</v>
       </c>
       <c r="F77" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="H77">
         <v>2</v>
       </c>
       <c r="I77" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="M77" t="s">
         <v>64</v>
@@ -5426,7 +5437,7 @@
         <v>1</v>
       </c>
       <c r="Z77" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="78" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -5434,10 +5445,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="C78" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="D78" t="s">
         <v>28</v>
@@ -5446,16 +5457,16 @@
         <v>130</v>
       </c>
       <c r="F78" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="H78">
         <v>1</v>
       </c>
       <c r="I78" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="M78" t="s">
         <v>212</v>
@@ -5475,7 +5486,7 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="C79" t="s">
         <v>156</v>
@@ -5487,16 +5498,16 @@
         <v>130</v>
       </c>
       <c r="F79" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="H79">
         <v>3</v>
       </c>
       <c r="I79" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="M79" t="s">
         <v>107</v>
@@ -5522,7 +5533,7 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="C80" t="s">
         <v>72</v>
@@ -5534,19 +5545,19 @@
         <v>130</v>
       </c>
       <c r="F80" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="H80">
         <v>3</v>
       </c>
       <c r="I80" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="J80" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="M80" t="s">
         <v>128</v>
@@ -5569,7 +5580,7 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="C81" t="s">
         <v>185</v>
@@ -5581,16 +5592,16 @@
         <v>130</v>
       </c>
       <c r="F81" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="H81">
         <v>2</v>
       </c>
       <c r="I81" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="M81" t="s">
         <v>128</v>
@@ -5610,10 +5621,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="C82" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="D82" t="s">
         <v>28</v>
@@ -5622,16 +5633,16 @@
         <v>130</v>
       </c>
       <c r="F82" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="H82">
         <v>2</v>
       </c>
       <c r="I82" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="83" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -5639,28 +5650,28 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="C83" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="D83" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="E83" t="s">
         <v>130</v>
       </c>
       <c r="F83" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>434</v>
+        <v>550</v>
       </c>
       <c r="H83">
         <v>3</v>
       </c>
       <c r="I83" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
     </row>
     <row r="84" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -5668,10 +5679,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="C84" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D84" t="s">
         <v>36</v>
@@ -5680,19 +5691,19 @@
         <v>130</v>
       </c>
       <c r="F84" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="H84">
         <v>1</v>
       </c>
       <c r="I84" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="J84" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="85" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -5700,7 +5711,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="C85" t="s">
         <v>109</v>
@@ -5712,19 +5723,19 @@
         <v>130</v>
       </c>
       <c r="F85" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="H85">
         <v>1</v>
       </c>
       <c r="I85" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="J85" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="86" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -5732,7 +5743,7 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="C86" t="s">
         <v>59</v>
@@ -5744,19 +5755,19 @@
         <v>130</v>
       </c>
       <c r="F86" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="H86">
         <v>2</v>
       </c>
       <c r="I86" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="J86" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="87" spans="1:26" ht="96" customHeight="1" x14ac:dyDescent="0.2">
@@ -5764,10 +5775,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="C87" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="D87" t="s">
         <v>36</v>
@@ -5776,19 +5787,19 @@
         <v>130</v>
       </c>
       <c r="F87" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="H87">
         <v>3</v>
       </c>
       <c r="I87" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="J87" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="88" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -5796,7 +5807,7 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="C88" t="s">
         <v>87</v>
@@ -5808,19 +5819,19 @@
         <v>130</v>
       </c>
       <c r="F88" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="H88">
         <v>1</v>
       </c>
       <c r="I88" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="J88" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="89" spans="1:26" ht="64" customHeight="1" x14ac:dyDescent="0.2">
@@ -5828,10 +5839,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="C89" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="D89" t="s">
         <v>36</v>
@@ -5840,19 +5851,19 @@
         <v>130</v>
       </c>
       <c r="F89" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="H89">
         <v>2</v>
       </c>
       <c r="I89" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="J89" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="90" spans="1:26" ht="64" customHeight="1" x14ac:dyDescent="0.2">
@@ -5860,10 +5871,10 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="C90" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D90" t="s">
         <v>36</v>
@@ -5872,16 +5883,16 @@
         <v>180</v>
       </c>
       <c r="F90" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="H90">
         <v>1</v>
       </c>
       <c r="I90" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="V90">
         <v>1</v>
@@ -5892,10 +5903,10 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="C91" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D91" t="s">
         <v>36</v>
@@ -5904,16 +5915,16 @@
         <v>180</v>
       </c>
       <c r="F91" t="s">
+        <v>460</v>
+      </c>
+      <c r="G91" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="G91" s="3" t="s">
-        <v>468</v>
-      </c>
       <c r="H91">
         <v>1</v>
       </c>
       <c r="I91" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="V91">
         <v>1</v>
@@ -5924,10 +5935,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="C92" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D92" t="s">
         <v>36</v>
@@ -5936,16 +5947,16 @@
         <v>180</v>
       </c>
       <c r="F92" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="H92">
         <v>2</v>
       </c>
       <c r="I92" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="T92">
         <v>1</v>
@@ -5959,10 +5970,10 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="C93" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="D93" t="s">
         <v>28</v>
@@ -5971,16 +5982,16 @@
         <v>180</v>
       </c>
       <c r="F93" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>477</v>
+        <v>553</v>
       </c>
       <c r="H93">
         <v>3</v>
       </c>
       <c r="I93" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="M93" t="s">
         <v>64</v>
@@ -5997,10 +6008,10 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="C94" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="D94" t="s">
         <v>36</v>
@@ -6009,16 +6020,16 @@
         <v>180</v>
       </c>
       <c r="F94" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="H94">
         <v>2</v>
       </c>
       <c r="I94" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="S94">
         <v>1</v>
@@ -6035,10 +6046,10 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="C95" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="D95" t="s">
         <v>36</v>
@@ -6047,16 +6058,16 @@
         <v>180</v>
       </c>
       <c r="F95" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="H95">
         <v>3</v>
       </c>
       <c r="I95" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="R95">
         <v>1</v>
@@ -6067,10 +6078,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="C96" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="D96" t="s">
         <v>36</v>
@@ -6079,16 +6090,16 @@
         <v>180</v>
       </c>
       <c r="F96" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="H96">
         <v>1</v>
       </c>
       <c r="I96" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="R96">
         <v>1</v>
@@ -6099,10 +6110,10 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="C97" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="D97" t="s">
         <v>36</v>
@@ -6111,16 +6122,16 @@
         <v>180</v>
       </c>
       <c r="F97" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="H97">
         <v>2</v>
       </c>
       <c r="I97" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="Q97">
         <v>1</v>
@@ -6137,10 +6148,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="C98" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="D98" t="s">
         <v>36</v>
@@ -6149,16 +6160,16 @@
         <v>180</v>
       </c>
       <c r="F98" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="H98">
         <v>1</v>
       </c>
       <c r="I98" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="S98">
         <v>1</v>
@@ -6172,7 +6183,7 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="C99" t="s">
         <v>244</v>
@@ -6184,16 +6195,16 @@
         <v>180</v>
       </c>
       <c r="F99" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>505</v>
+        <v>552</v>
       </c>
       <c r="H99">
         <v>2</v>
       </c>
       <c r="I99" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="M99" t="s">
         <v>107</v>
@@ -6210,10 +6221,10 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="C100" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D100" t="s">
         <v>36</v>
@@ -6222,19 +6233,19 @@
         <v>180</v>
       </c>
       <c r="F100" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="H100">
         <v>2</v>
       </c>
       <c r="I100" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="J100" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="101" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -6242,10 +6253,10 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="C101" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D101" t="s">
         <v>28</v>
@@ -6254,16 +6265,16 @@
         <v>180</v>
       </c>
       <c r="F101" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="H101">
         <v>3</v>
       </c>
       <c r="I101" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
     </row>
     <row r="102" spans="1:24" ht="144" customHeight="1" x14ac:dyDescent="0.2">
@@ -6271,10 +6282,10 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
       <c r="C102" t="s">
-        <v>516</v>
+        <v>510</v>
       </c>
       <c r="D102" t="s">
         <v>36</v>
@@ -6283,19 +6294,19 @@
         <v>180</v>
       </c>
       <c r="F102" t="s">
-        <v>517</v>
+        <v>511</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="H102">
         <v>1</v>
       </c>
       <c r="I102" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="J102" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="103" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -6303,10 +6314,10 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="C103" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="D103" t="s">
         <v>36</v>
@@ -6315,16 +6326,16 @@
         <v>180</v>
       </c>
       <c r="F103" t="s">
-        <v>521</v>
+        <v>515</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>522</v>
+        <v>516</v>
       </c>
       <c r="H103">
         <v>1</v>
       </c>
       <c r="I103" t="s">
-        <v>523</v>
+        <v>517</v>
       </c>
       <c r="V103">
         <v>1</v>
@@ -6335,7 +6346,7 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>524</v>
+        <v>518</v>
       </c>
       <c r="C104" t="s">
         <v>235</v>
@@ -6347,16 +6358,16 @@
         <v>180</v>
       </c>
       <c r="F104" t="s">
-        <v>525</v>
+        <v>519</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
       <c r="H104">
         <v>3</v>
       </c>
       <c r="I104" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
       <c r="S104">
         <v>1</v>
@@ -6370,10 +6381,10 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>528</v>
+        <v>522</v>
       </c>
       <c r="C105" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D105" t="s">
         <v>28</v>
@@ -6382,19 +6393,19 @@
         <v>180</v>
       </c>
       <c r="F105" t="s">
-        <v>529</v>
+        <v>523</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>530</v>
+        <v>524</v>
       </c>
       <c r="H105">
         <v>3</v>
       </c>
       <c r="I105" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="J105" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="106" spans="1:24" ht="64" customHeight="1" x14ac:dyDescent="0.2">
@@ -6402,10 +6413,10 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>532</v>
+        <v>526</v>
       </c>
       <c r="C106" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="D106" t="s">
         <v>36</v>
@@ -6414,19 +6425,19 @@
         <v>180</v>
       </c>
       <c r="F106" t="s">
-        <v>534</v>
+        <v>528</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="H106">
         <v>2</v>
       </c>
       <c r="I106" t="s">
-        <v>536</v>
+        <v>530</v>
       </c>
       <c r="J106" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="107" spans="1:24" ht="64" customHeight="1" x14ac:dyDescent="0.2">
@@ -6434,10 +6445,10 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
       <c r="C107" t="s">
-        <v>538</v>
+        <v>532</v>
       </c>
       <c r="D107" t="s">
         <v>28</v>
@@ -6446,19 +6457,19 @@
         <v>180</v>
       </c>
       <c r="F107" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="H107">
         <v>1</v>
       </c>
       <c r="I107" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="J107" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="108" spans="1:24" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -6466,10 +6477,10 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="C108" t="s">
-        <v>538</v>
+        <v>532</v>
       </c>
       <c r="D108" t="s">
         <v>28</v>
@@ -6478,19 +6489,19 @@
         <v>180</v>
       </c>
       <c r="F108" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="H108">
         <v>1</v>
       </c>
       <c r="I108" t="s">
-        <v>545</v>
+        <v>539</v>
       </c>
       <c r="J108" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="109" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -6498,10 +6509,10 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="C109" t="s">
-        <v>547</v>
+        <v>541</v>
       </c>
       <c r="D109" t="s">
         <v>36</v>
@@ -6510,19 +6521,19 @@
         <v>180</v>
       </c>
       <c r="F109" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="H109">
         <v>1</v>
       </c>
       <c r="I109" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="J109" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="110" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -6530,31 +6541,34 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="C110" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="E110" t="s">
         <v>180</v>
       </c>
       <c r="F110" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="H110">
         <v>2</v>
       </c>
       <c r="I110" t="s">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="J110" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;KFF8C00 CONFIDENTIAL&amp;1#_x000D_</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
GBA: more bug fix. new: tourfontaine impelmeentation.
</commit_message>
<xml_diff>
--- a/src/resources/horde_cards.xlsx
+++ b/src/resources/horde_cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dsaban/git/perso/windwalkers-cardgame/src/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF051C5A-07D0-7245-AC65-4AC170CD20A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E170C1-EA41-FD4E-96A6-0F9211AD5D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-140" yWindow="1160" windowWidth="28920" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="940" windowWidth="28920" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2104,8 +2104,11 @@
   <dimension ref="A1:Z110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="20.6640625" customWidth="1"/>
-    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" customWidth="1"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.6640625" customWidth="1"/>
+    <col min="5" max="5" width="7.33203125" customWidth="1"/>
     <col min="7" max="7" width="26.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6567,6 +6570,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <headerFooter>
     <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;KFF8C00 CONFIDENTIAL&amp;1#_x000D_</oddHeader>
   </headerFooter>

</xml_diff>